<commit_message>
Update aviation page with latest Fly.xlsx records
</commit_message>
<xml_diff>
--- a/files/Fly.xlsx
+++ b/files/Fly.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="588" uniqueCount="323">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="338">
   <si>
     <t>Date</t>
   </si>
@@ -996,6 +996,51 @@
   </si>
   <si>
     <t>31A</t>
+  </si>
+  <si>
+    <t>MU5622</t>
+  </si>
+  <si>
+    <t>B32NL</t>
+  </si>
+  <si>
+    <t>7812211250146</t>
+  </si>
+  <si>
+    <t>MU6221</t>
+  </si>
+  <si>
+    <t>KHG</t>
+  </si>
+  <si>
+    <t>B325U</t>
+  </si>
+  <si>
+    <t>54A</t>
+  </si>
+  <si>
+    <t>CZ8891</t>
+  </si>
+  <si>
+    <t>PKX</t>
+  </si>
+  <si>
+    <t>B1238</t>
+  </si>
+  <si>
+    <t>67K</t>
+  </si>
+  <si>
+    <t>7842172724860</t>
+  </si>
+  <si>
+    <t>CZ6122</t>
+  </si>
+  <si>
+    <t>B6580</t>
+  </si>
+  <si>
+    <t>49A</t>
   </si>
 </sst>
 </file>
@@ -1009,10 +1054,25 @@
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="176" formatCode="h:mm;@"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -1162,12 +1222,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -1482,137 +1548,137 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1628,13 +1694,88 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="176" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2162,7 +2303,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:K70"/>
+  <dimension ref="A1:K74"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="1" width="10.8046875" style="1" customWidth="1"/>
@@ -2197,7 +2338,7 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="17" t="s">
         <v>7</v>
       </c>
       <c r="I1" s="2" t="s">
@@ -2206,7 +2347,7 @@
       <c r="J1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="K1" s="17" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2232,16 +2373,16 @@
       <c r="G2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="I2" s="7" t="s">
+      <c r="I2" s="29" t="s">
         <v>18</v>
       </c>
       <c r="J2" s="3">
         <v>1074</v>
       </c>
-      <c r="K2" s="5">
+      <c r="K2" s="17">
         <v>0.0611111111111111</v>
       </c>
     </row>
@@ -2267,16 +2408,16 @@
       <c r="G3" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H3" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="I3" s="7" t="s">
+      <c r="I3" s="29" t="s">
         <v>18</v>
       </c>
       <c r="J3" s="3">
         <v>1074</v>
       </c>
-      <c r="K3" s="5">
+      <c r="K3" s="17">
         <v>0.06875</v>
       </c>
     </row>
@@ -2302,16 +2443,16 @@
       <c r="G4" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="H4" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="I4" s="7" t="s">
+      <c r="I4" s="29" t="s">
         <v>25</v>
       </c>
       <c r="J4" s="3">
         <v>1074</v>
       </c>
-      <c r="K4" s="5">
+      <c r="K4" s="17">
         <v>0.0590277777777778</v>
       </c>
     </row>
@@ -2337,51 +2478,51 @@
       <c r="G5" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="H5" s="5" t="s">
+      <c r="H5" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="I5" s="7" t="s">
+      <c r="I5" s="29" t="s">
         <v>25</v>
       </c>
       <c r="J5" s="3">
         <v>1074</v>
       </c>
-      <c r="K5" s="5">
+      <c r="K5" s="17">
         <v>0.0708333333333333</v>
       </c>
     </row>
     <row r="6" spans="1:11">
-      <c r="A6" s="4">
+      <c r="A6" s="5">
         <v>43629</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E6" s="1" t="s">
+      <c r="D6" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="G6" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="H6" s="5" t="s">
+      <c r="H6" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="I6" s="7" t="s">
+      <c r="I6" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="J6" s="3">
+      <c r="J6" s="20">
         <v>1419</v>
       </c>
-      <c r="K6" s="5">
+      <c r="K6" s="18">
         <v>0.0881944444444444</v>
       </c>
     </row>
@@ -2407,16 +2548,16 @@
       <c r="G7" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="H7" s="5" t="s">
+      <c r="H7" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="I7" s="7" t="s">
+      <c r="I7" s="29" t="s">
         <v>40</v>
       </c>
       <c r="J7" s="3">
         <v>323</v>
       </c>
-      <c r="K7" s="5">
+      <c r="K7" s="17">
         <v>0.0256944444444444</v>
       </c>
     </row>
@@ -2442,16 +2583,16 @@
       <c r="G8" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="H8" s="5" t="s">
+      <c r="H8" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="I8" s="7" t="s">
+      <c r="I8" s="29" t="s">
         <v>45</v>
       </c>
       <c r="J8" s="3">
         <v>323</v>
       </c>
-      <c r="K8" s="5">
+      <c r="K8" s="17">
         <v>0.0298611111111111</v>
       </c>
     </row>
@@ -2477,16 +2618,16 @@
       <c r="G9" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="H9" s="5" t="s">
+      <c r="H9" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="I9" s="7" t="s">
+      <c r="I9" s="29" t="s">
         <v>49</v>
       </c>
       <c r="J9" s="3">
         <v>323</v>
       </c>
-      <c r="K9" s="5">
+      <c r="K9" s="17">
         <v>0.0263888888888889</v>
       </c>
     </row>
@@ -2512,16 +2653,16 @@
       <c r="G10" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="H10" s="5" t="s">
+      <c r="H10" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="I10" s="7" t="s">
+      <c r="I10" s="29" t="s">
         <v>52</v>
       </c>
       <c r="J10" s="3">
         <v>323</v>
       </c>
-      <c r="K10" s="5">
+      <c r="K10" s="17">
         <v>0.0298611111111111</v>
       </c>
     </row>
@@ -2547,16 +2688,16 @@
       <c r="G11" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="H11" s="5" t="s">
+      <c r="H11" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="I11" s="7" t="s">
+      <c r="I11" s="29" t="s">
         <v>56</v>
       </c>
       <c r="J11" s="3">
         <v>323</v>
       </c>
-      <c r="K11" s="5">
+      <c r="K11" s="17">
         <v>0.0263888888888889</v>
       </c>
     </row>
@@ -2582,16 +2723,16 @@
       <c r="G12" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="H12" s="5" t="s">
+      <c r="H12" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="I12" s="7" t="s">
+      <c r="I12" s="29" t="s">
         <v>59</v>
       </c>
       <c r="J12" s="3">
         <v>323</v>
       </c>
-      <c r="K12" s="5">
+      <c r="K12" s="17">
         <v>0.03125</v>
       </c>
     </row>
@@ -2617,16 +2758,16 @@
       <c r="G13" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="H13" s="5" t="s">
+      <c r="H13" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="I13" s="7" t="s">
+      <c r="I13" s="29" t="s">
         <v>62</v>
       </c>
       <c r="J13" s="3">
         <v>323</v>
       </c>
-      <c r="K13" s="5">
+      <c r="K13" s="17">
         <v>0.0263888888888889</v>
       </c>
     </row>
@@ -2652,16 +2793,16 @@
       <c r="G14" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="H14" s="5" t="s">
+      <c r="H14" s="17" t="s">
         <v>67</v>
       </c>
-      <c r="I14" s="7" t="s">
+      <c r="I14" s="29" t="s">
         <v>68</v>
       </c>
       <c r="J14" s="3">
         <v>1664</v>
       </c>
-      <c r="K14" s="5">
+      <c r="K14" s="17">
         <v>0.114583333333333</v>
       </c>
     </row>
@@ -2687,16 +2828,16 @@
       <c r="G15" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="H15" s="5" t="s">
+      <c r="H15" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="I15" s="7" t="s">
+      <c r="I15" s="29" t="s">
         <v>74</v>
       </c>
       <c r="J15" s="3">
         <v>603</v>
       </c>
-      <c r="K15" s="5">
+      <c r="K15" s="17">
         <v>0.0361111111111111</v>
       </c>
     </row>
@@ -2722,16 +2863,16 @@
       <c r="G16" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="H16" s="5" t="s">
+      <c r="H16" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="I16" s="7" t="s">
+      <c r="I16" s="29" t="s">
         <v>80</v>
       </c>
       <c r="J16" s="3">
         <v>1228</v>
       </c>
-      <c r="K16" s="5">
+      <c r="K16" s="17">
         <v>0.0875</v>
       </c>
     </row>
@@ -2757,16 +2898,16 @@
       <c r="G17" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="H17" s="5" t="s">
+      <c r="H17" s="17" t="s">
         <v>85</v>
       </c>
-      <c r="I17" s="7" t="s">
+      <c r="I17" s="29" t="s">
         <v>86</v>
       </c>
       <c r="J17" s="3">
         <v>358</v>
       </c>
-      <c r="K17" s="5">
+      <c r="K17" s="17">
         <v>0.0381944444444444</v>
       </c>
     </row>
@@ -2792,51 +2933,51 @@
       <c r="G18" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="H18" s="5" t="s">
+      <c r="H18" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="I18" s="7" t="s">
+      <c r="I18" s="29" t="s">
         <v>91</v>
       </c>
       <c r="J18" s="3">
         <v>1460</v>
       </c>
-      <c r="K18" s="5">
+      <c r="K18" s="17">
         <v>0.0875</v>
       </c>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="4">
+      <c r="A19" s="8">
         <v>45368</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C19" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="D19" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E19" s="1" t="s">
+      <c r="D19" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E19" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="F19" s="1" t="s">
+      <c r="F19" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="G19" s="1" t="s">
+      <c r="G19" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="H19" s="5" t="s">
+      <c r="H19" s="19" t="s">
         <v>95</v>
       </c>
-      <c r="I19" s="7" t="s">
+      <c r="I19" s="31" t="s">
         <v>96</v>
       </c>
-      <c r="J19" s="3">
+      <c r="J19" s="21">
         <v>1460</v>
       </c>
-      <c r="K19" s="5">
+      <c r="K19" s="19">
         <v>0.0770833333333333</v>
       </c>
     </row>
@@ -2862,86 +3003,86 @@
       <c r="G20" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="H20" s="5" t="s">
+      <c r="H20" s="17" t="s">
         <v>85</v>
       </c>
-      <c r="I20" s="7" t="s">
+      <c r="I20" s="29" t="s">
         <v>99</v>
       </c>
       <c r="J20" s="3">
         <v>1051</v>
       </c>
-      <c r="K20" s="5">
+      <c r="K20" s="17">
         <v>0.0659722222222222</v>
       </c>
     </row>
     <row r="21" spans="1:11">
-      <c r="A21" s="4">
+      <c r="A21" s="11">
         <v>45422</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="C21" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="D21" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E21" s="1" t="s">
+      <c r="D21" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="E21" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="F21" s="1" t="s">
+      <c r="F21" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="G21" s="1" t="s">
+      <c r="G21" s="12" t="s">
         <v>103</v>
       </c>
-      <c r="H21" s="1" t="s">
+      <c r="H21" s="12" t="s">
         <v>104</v>
       </c>
-      <c r="I21" s="7" t="s">
+      <c r="I21" s="32" t="s">
         <v>99</v>
       </c>
-      <c r="J21" s="3">
+      <c r="J21" s="22">
         <v>3796</v>
       </c>
-      <c r="K21" s="6">
+      <c r="K21" s="23">
         <v>0.206944444444444</v>
       </c>
     </row>
     <row r="22" spans="1:11">
-      <c r="A22" s="4">
+      <c r="A22" s="11">
         <v>45428</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B22" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="C22" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="D22" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E22" s="1" t="s">
+      <c r="D22" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="E22" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="F22" s="1" t="s">
+      <c r="F22" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="G22" s="1" t="s">
+      <c r="G22" s="12" t="s">
         <v>107</v>
       </c>
-      <c r="H22" s="1" t="s">
+      <c r="H22" s="12" t="s">
         <v>108</v>
       </c>
-      <c r="I22" s="2" t="s">
+      <c r="I22" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="J22" s="3" t="s">
+      <c r="J22" s="22" t="s">
         <v>109</v>
       </c>
-      <c r="K22" s="6">
+      <c r="K22" s="23">
         <v>0.200694444444444</v>
       </c>
     </row>
@@ -2976,7 +3117,7 @@
       <c r="J23" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="K23" s="6">
+      <c r="K23" s="24">
         <v>0.0680555555555555</v>
       </c>
     </row>
@@ -3011,7 +3152,7 @@
       <c r="J24" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="K24" s="6">
+      <c r="K24" s="24">
         <v>0.03125</v>
       </c>
     </row>
@@ -3046,112 +3187,112 @@
       <c r="J25" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="K25" s="6">
+      <c r="K25" s="24">
         <v>0.0263888888888889</v>
       </c>
     </row>
     <row r="26" spans="1:11">
-      <c r="A26" s="4">
+      <c r="A26" s="14">
         <v>45462</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B26" s="15" t="s">
         <v>122</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="C26" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="D26" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E26" s="1" t="s">
+      <c r="D26" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="E26" s="15" t="s">
         <v>123</v>
       </c>
-      <c r="F26" s="1" t="s">
+      <c r="F26" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="G26" s="1" t="s">
+      <c r="G26" s="15" t="s">
         <v>124</v>
       </c>
-      <c r="H26" s="1" t="s">
+      <c r="H26" s="15" t="s">
         <v>125</v>
       </c>
-      <c r="I26" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="J26" s="3" t="s">
+      <c r="I26" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="J26" s="25" t="s">
         <v>126</v>
       </c>
-      <c r="K26" s="6">
+      <c r="K26" s="26">
         <v>0.0868055555555556</v>
       </c>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="4">
+      <c r="A27" s="14">
         <v>45466</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B27" s="15" t="s">
         <v>127</v>
       </c>
-      <c r="C27" s="1" t="s">
+      <c r="C27" s="15" t="s">
         <v>123</v>
       </c>
-      <c r="D27" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E27" s="1" t="s">
+      <c r="D27" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="E27" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="F27" s="1" t="s">
+      <c r="F27" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="G27" s="1" t="s">
+      <c r="G27" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="H27" s="1" t="s">
+      <c r="H27" s="15" t="s">
         <v>129</v>
       </c>
-      <c r="I27" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="J27" s="3" t="s">
+      <c r="I27" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="J27" s="25" t="s">
         <v>126</v>
       </c>
-      <c r="K27" s="6">
+      <c r="K27" s="26">
         <v>0.0888888888888889</v>
       </c>
     </row>
     <row r="28" spans="1:11">
-      <c r="A28" s="4">
+      <c r="A28" s="8">
         <v>45488</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B28" s="9" t="s">
         <v>130</v>
       </c>
-      <c r="C28" s="1" t="s">
+      <c r="C28" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D28" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E28" s="1" t="s">
+      <c r="D28" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E28" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="F28" s="1" t="s">
+      <c r="F28" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="G28" s="1" t="s">
+      <c r="G28" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="H28" s="1" t="s">
+      <c r="H28" s="9" t="s">
         <v>133</v>
       </c>
-      <c r="I28" s="2" t="s">
+      <c r="I28" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="J28" s="3" t="s">
+      <c r="J28" s="21" t="s">
         <v>135</v>
       </c>
-      <c r="K28" s="6">
+      <c r="K28" s="27">
         <v>0.0361111111111111</v>
       </c>
     </row>
@@ -3186,7 +3327,7 @@
       <c r="J29" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="K29" s="6">
+      <c r="K29" s="24">
         <v>0.0652777777777778</v>
       </c>
     </row>
@@ -3221,7 +3362,7 @@
       <c r="J30" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="K30" s="6">
+      <c r="K30" s="24">
         <v>0.0534722222222222</v>
       </c>
     </row>
@@ -3256,7 +3397,7 @@
       <c r="J31" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="K31" s="6">
+      <c r="K31" s="24">
         <v>0.09375</v>
       </c>
     </row>
@@ -3291,7 +3432,7 @@
       <c r="J32" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="K32" s="6">
+      <c r="K32" s="24">
         <v>0.0430555555555556</v>
       </c>
     </row>
@@ -3326,7 +3467,7 @@
       <c r="J33" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="K33" s="6">
+      <c r="K33" s="24">
         <v>0.0451388888888889</v>
       </c>
     </row>
@@ -3361,7 +3502,7 @@
       <c r="J34" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="K34" s="6">
+      <c r="K34" s="24">
         <v>0.0381944444444444</v>
       </c>
     </row>
@@ -3396,7 +3537,7 @@
       <c r="J35" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="K35" s="6">
+      <c r="K35" s="24">
         <v>0.0805555555555556</v>
       </c>
     </row>
@@ -3431,7 +3572,7 @@
       <c r="J36" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="K36" s="6">
+      <c r="K36" s="24">
         <v>0.0645833333333333</v>
       </c>
     </row>
@@ -3466,7 +3607,7 @@
       <c r="J37" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="K37" s="6">
+      <c r="K37" s="24">
         <v>0.0319444444444444</v>
       </c>
     </row>
@@ -3501,7 +3642,7 @@
       <c r="J38" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="K38" s="6">
+      <c r="K38" s="24">
         <v>0.0513888888888889</v>
       </c>
     </row>
@@ -3536,7 +3677,7 @@
       <c r="J39" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="K39" s="6">
+      <c r="K39" s="24">
         <v>0.0638888888888889</v>
       </c>
     </row>
@@ -3571,7 +3712,7 @@
       <c r="J40" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="K40" s="6">
+      <c r="K40" s="24">
         <v>0.0729166666666667</v>
       </c>
     </row>
@@ -3606,322 +3747,322 @@
       <c r="J41" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="K41" s="6">
+      <c r="K41" s="24">
         <v>0.0291666666666667</v>
       </c>
     </row>
     <row r="42" spans="1:11">
-      <c r="A42" s="4">
+      <c r="A42" s="8">
         <v>45705</v>
       </c>
-      <c r="B42" s="1" t="s">
+      <c r="B42" s="9" t="s">
         <v>201</v>
       </c>
-      <c r="C42" s="1" t="s">
+      <c r="C42" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="D42" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E42" s="1" t="s">
+      <c r="D42" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E42" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="F42" s="1" t="s">
+      <c r="F42" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="G42" s="1" t="s">
+      <c r="G42" s="9" t="s">
         <v>202</v>
       </c>
-      <c r="H42" s="1" t="s">
+      <c r="H42" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="I42" s="2" t="s">
+      <c r="I42" s="10" t="s">
         <v>203</v>
       </c>
-      <c r="J42" s="3" t="s">
+      <c r="J42" s="21" t="s">
         <v>135</v>
       </c>
-      <c r="K42" s="6">
+      <c r="K42" s="27">
         <v>0.0416666666666667</v>
       </c>
     </row>
     <row r="43" spans="1:11">
-      <c r="A43" s="4">
+      <c r="A43" s="14">
         <v>45708</v>
       </c>
-      <c r="B43" s="1" t="s">
+      <c r="B43" s="15" t="s">
         <v>204</v>
       </c>
-      <c r="C43" s="1" t="s">
+      <c r="C43" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="D43" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E43" s="1" t="s">
+      <c r="D43" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="E43" s="15" t="s">
         <v>205</v>
       </c>
-      <c r="F43" s="1" t="s">
+      <c r="F43" s="15" t="s">
         <v>206</v>
       </c>
-      <c r="G43" s="1" t="s">
+      <c r="G43" s="15" t="s">
         <v>207</v>
       </c>
-      <c r="H43" s="1" t="s">
+      <c r="H43" s="15" t="s">
         <v>208</v>
       </c>
-      <c r="I43" s="2" t="s">
+      <c r="I43" s="16" t="s">
         <v>209</v>
       </c>
-      <c r="J43" s="3" t="s">
+      <c r="J43" s="25" t="s">
         <v>210</v>
       </c>
-      <c r="K43" s="6">
+      <c r="K43" s="26">
         <v>0.0375</v>
       </c>
     </row>
     <row r="44" spans="1:11">
-      <c r="A44" s="4">
+      <c r="A44" s="11">
         <v>45708</v>
       </c>
-      <c r="B44" s="1" t="s">
+      <c r="B44" s="12" t="s">
         <v>211</v>
       </c>
-      <c r="C44" s="1" t="s">
+      <c r="C44" s="12" t="s">
         <v>205</v>
       </c>
-      <c r="D44" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E44" s="1" t="s">
+      <c r="D44" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="E44" s="12" t="s">
         <v>212</v>
       </c>
-      <c r="F44" s="1" t="s">
+      <c r="F44" s="12" t="s">
         <v>213</v>
       </c>
-      <c r="G44" s="1" t="s">
+      <c r="G44" s="12" t="s">
         <v>214</v>
       </c>
-      <c r="H44" s="1" t="s">
+      <c r="H44" s="12" t="s">
         <v>215</v>
       </c>
-      <c r="I44" s="2" t="s">
+      <c r="I44" s="13" t="s">
         <v>209</v>
       </c>
-      <c r="J44" s="3" t="s">
+      <c r="J44" s="22" t="s">
         <v>216</v>
       </c>
-      <c r="K44" s="6">
+      <c r="K44" s="23">
         <v>0.413888888888889</v>
       </c>
     </row>
     <row r="45" spans="1:11">
-      <c r="A45" s="4">
+      <c r="A45" s="14">
         <v>45711</v>
       </c>
-      <c r="B45" s="1" t="s">
+      <c r="B45" s="15" t="s">
         <v>217</v>
       </c>
-      <c r="C45" s="1" t="s">
+      <c r="C45" s="15" t="s">
         <v>212</v>
       </c>
-      <c r="D45" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E45" s="1" t="s">
+      <c r="D45" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="E45" s="15" t="s">
         <v>218</v>
       </c>
-      <c r="F45" s="1" t="s">
+      <c r="F45" s="15" t="s">
         <v>219</v>
       </c>
-      <c r="G45" s="1" t="s">
+      <c r="G45" s="15" t="s">
         <v>220</v>
       </c>
-      <c r="H45" s="1" t="s">
+      <c r="H45" s="15" t="s">
         <v>221</v>
       </c>
-      <c r="I45" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="J45" s="3" t="s">
+      <c r="I45" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="J45" s="25" t="s">
         <v>222</v>
       </c>
-      <c r="K45" s="6">
+      <c r="K45" s="26">
         <v>0.0347222222222222</v>
       </c>
     </row>
     <row r="46" spans="1:11">
-      <c r="A46" s="4">
+      <c r="A46" s="14">
         <v>45712</v>
       </c>
-      <c r="B46" s="1" t="s">
+      <c r="B46" s="15" t="s">
         <v>223</v>
       </c>
-      <c r="C46" s="1" t="s">
+      <c r="C46" s="15" t="s">
         <v>218</v>
       </c>
-      <c r="D46" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E46" s="1" t="s">
+      <c r="D46" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="E46" s="15" t="s">
         <v>224</v>
       </c>
-      <c r="F46" s="1" t="s">
+      <c r="F46" s="15" t="s">
         <v>206</v>
       </c>
-      <c r="G46" s="1" t="s">
+      <c r="G46" s="15" t="s">
         <v>225</v>
       </c>
-      <c r="H46" s="1" t="s">
+      <c r="H46" s="15" t="s">
         <v>226</v>
       </c>
-      <c r="I46" s="2" t="s">
+      <c r="I46" s="16" t="s">
         <v>227</v>
       </c>
-      <c r="J46" s="3" t="s">
+      <c r="J46" s="25" t="s">
         <v>228</v>
       </c>
-      <c r="K46" s="6">
+      <c r="K46" s="26">
         <v>0.198611111111111</v>
       </c>
     </row>
     <row r="47" spans="1:11">
-      <c r="A47" s="4">
+      <c r="A47" s="14">
         <v>45715</v>
       </c>
-      <c r="B47" s="1" t="s">
+      <c r="B47" s="15" t="s">
         <v>229</v>
       </c>
-      <c r="C47" s="1" t="s">
+      <c r="C47" s="15" t="s">
         <v>224</v>
       </c>
-      <c r="D47" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E47" s="1" t="s">
+      <c r="D47" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="E47" s="15" t="s">
         <v>230</v>
       </c>
-      <c r="F47" s="1" t="s">
+      <c r="F47" s="15" t="s">
         <v>231</v>
       </c>
-      <c r="G47" s="1" t="s">
+      <c r="G47" s="15" t="s">
         <v>232</v>
       </c>
-      <c r="H47" s="1" t="s">
+      <c r="H47" s="15" t="s">
         <v>233</v>
       </c>
-      <c r="I47" s="2" t="s">
+      <c r="I47" s="16" t="s">
         <v>234</v>
       </c>
-      <c r="J47" s="3">
+      <c r="J47" s="25">
         <v>342</v>
       </c>
-      <c r="K47" s="6">
+      <c r="K47" s="26">
         <v>0.0409722222222222</v>
       </c>
     </row>
     <row r="48" spans="1:11">
-      <c r="A48" s="4">
+      <c r="A48" s="14">
         <v>45717</v>
       </c>
-      <c r="B48" s="1" t="s">
+      <c r="B48" s="15" t="s">
         <v>235</v>
       </c>
-      <c r="C48" s="1" t="s">
+      <c r="C48" s="15" t="s">
         <v>230</v>
       </c>
-      <c r="D48" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E48" s="1" t="s">
+      <c r="D48" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="E48" s="15" t="s">
         <v>212</v>
       </c>
-      <c r="F48" s="1" t="s">
+      <c r="F48" s="15" t="s">
         <v>236</v>
       </c>
-      <c r="G48" s="1" t="s">
+      <c r="G48" s="15" t="s">
         <v>237</v>
       </c>
-      <c r="H48" s="1" t="s">
+      <c r="H48" s="15" t="s">
         <v>238</v>
       </c>
-      <c r="I48" s="2" t="s">
+      <c r="I48" s="16" t="s">
         <v>239</v>
       </c>
-      <c r="J48" s="3">
+      <c r="J48" s="25">
         <v>3714</v>
       </c>
-      <c r="K48" s="6">
+      <c r="K48" s="26">
         <v>0.211805555555556</v>
       </c>
     </row>
     <row r="49" spans="1:11">
-      <c r="A49" s="4">
+      <c r="A49" s="11">
         <v>45718</v>
       </c>
-      <c r="B49" s="1" t="s">
+      <c r="B49" s="12" t="s">
         <v>240</v>
       </c>
-      <c r="C49" s="1" t="s">
+      <c r="C49" s="12" t="s">
         <v>212</v>
       </c>
-      <c r="D49" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E49" s="1" t="s">
+      <c r="D49" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="E49" s="12" t="s">
         <v>205</v>
       </c>
-      <c r="F49" s="1" t="s">
+      <c r="F49" s="12" t="s">
         <v>241</v>
       </c>
-      <c r="G49" s="1" t="s">
+      <c r="G49" s="12" t="s">
         <v>242</v>
       </c>
-      <c r="H49" s="1" t="s">
+      <c r="H49" s="12" t="s">
         <v>243</v>
       </c>
-      <c r="I49" s="2" t="s">
+      <c r="I49" s="13" t="s">
         <v>209</v>
       </c>
-      <c r="J49" s="3">
+      <c r="J49" s="22">
         <v>9612</v>
       </c>
-      <c r="K49" s="6">
+      <c r="K49" s="23">
         <v>0.534722222222222</v>
       </c>
     </row>
     <row r="50" spans="1:11">
-      <c r="A50" s="4">
+      <c r="A50" s="14">
         <v>45720</v>
       </c>
-      <c r="B50" s="1" t="s">
+      <c r="B50" s="15" t="s">
         <v>244</v>
       </c>
-      <c r="C50" s="1" t="s">
+      <c r="C50" s="15" t="s">
         <v>205</v>
       </c>
-      <c r="D50" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E50" s="1" t="s">
+      <c r="D50" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="E50" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="F50" s="1" t="s">
+      <c r="F50" s="15" t="s">
         <v>206</v>
       </c>
-      <c r="G50" s="1" t="s">
+      <c r="G50" s="15" t="s">
         <v>245</v>
       </c>
-      <c r="H50" s="1" t="s">
+      <c r="H50" s="15" t="s">
         <v>246</v>
       </c>
-      <c r="I50" s="2" t="s">
+      <c r="I50" s="16" t="s">
         <v>209</v>
       </c>
-      <c r="J50" s="3">
+      <c r="J50" s="25">
         <v>460</v>
       </c>
-      <c r="K50" s="6">
+      <c r="K50" s="26">
         <v>0.0395833333333333</v>
       </c>
     </row>
@@ -3956,7 +4097,7 @@
       <c r="J51" s="3">
         <v>1194</v>
       </c>
-      <c r="K51" s="6">
+      <c r="K51" s="24">
         <v>0.0611111111111111</v>
       </c>
     </row>
@@ -3991,7 +4132,7 @@
       <c r="J52" s="3">
         <v>1194</v>
       </c>
-      <c r="K52" s="6">
+      <c r="K52" s="24">
         <v>0.05</v>
       </c>
     </row>
@@ -4026,7 +4167,7 @@
       <c r="J53" s="3">
         <v>670</v>
       </c>
-      <c r="K53" s="6">
+      <c r="K53" s="24">
         <v>0.0347222222222222</v>
       </c>
     </row>
@@ -4061,7 +4202,7 @@
       <c r="J54" s="3">
         <v>670</v>
       </c>
-      <c r="K54" s="6">
+      <c r="K54" s="24">
         <v>0.0381944444444444</v>
       </c>
     </row>
@@ -4096,42 +4237,42 @@
       <c r="J55" s="3">
         <v>670</v>
       </c>
-      <c r="K55" s="6">
+      <c r="K55" s="24">
         <v>0.0416666666666667</v>
       </c>
     </row>
     <row r="56" spans="1:11">
-      <c r="A56" s="4">
+      <c r="A56" s="8">
         <v>45940</v>
       </c>
-      <c r="B56" s="1" t="s">
+      <c r="B56" s="9" t="s">
         <v>268</v>
       </c>
-      <c r="C56" s="1" t="s">
+      <c r="C56" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="D56" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E56" s="1" t="s">
+      <c r="D56" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E56" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="F56" s="1" t="s">
+      <c r="F56" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="G56" s="1" t="s">
+      <c r="G56" s="9" t="s">
         <v>269</v>
       </c>
-      <c r="H56" s="1" t="s">
+      <c r="H56" s="9" t="s">
         <v>270</v>
       </c>
-      <c r="I56" s="2" t="s">
+      <c r="I56" s="10" t="s">
         <v>271</v>
       </c>
-      <c r="J56" s="3">
+      <c r="J56" s="21">
         <v>670</v>
       </c>
-      <c r="K56" s="6">
+      <c r="K56" s="27">
         <v>0.0354166666666667</v>
       </c>
     </row>
@@ -4166,7 +4307,7 @@
       <c r="J57" s="3">
         <v>2368</v>
       </c>
-      <c r="K57" s="6">
+      <c r="K57" s="24">
         <v>0.136805555555556</v>
       </c>
     </row>
@@ -4201,7 +4342,7 @@
       <c r="J58" s="3">
         <v>2285</v>
       </c>
-      <c r="K58" s="6">
+      <c r="K58" s="24">
         <v>0.189583333333333</v>
       </c>
     </row>
@@ -4236,7 +4377,7 @@
       <c r="J59" s="3">
         <v>1051</v>
       </c>
-      <c r="K59" s="6">
+      <c r="K59" s="24">
         <v>0.0777777777777778</v>
       </c>
     </row>
@@ -4271,7 +4412,7 @@
       <c r="J60" s="3">
         <v>1184</v>
       </c>
-      <c r="K60" s="6">
+      <c r="K60" s="24">
         <v>0.0590277777777778</v>
       </c>
     </row>
@@ -4306,7 +4447,7 @@
       <c r="J61" s="3">
         <v>1918</v>
       </c>
-      <c r="K61" s="6">
+      <c r="K61" s="24">
         <v>0.171527777777778</v>
       </c>
     </row>
@@ -4341,42 +4482,42 @@
       <c r="J62" s="3">
         <v>940</v>
       </c>
-      <c r="K62" s="6">
+      <c r="K62" s="24">
         <v>0.0534722222222222</v>
       </c>
     </row>
     <row r="63" spans="1:11">
-      <c r="A63" s="4">
+      <c r="A63" s="5">
         <v>46029</v>
       </c>
-      <c r="B63" s="1" t="s">
+      <c r="B63" s="6" t="s">
         <v>293</v>
       </c>
-      <c r="C63" s="1" t="s">
+      <c r="C63" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="D63" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E63" s="1" t="s">
+      <c r="D63" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E63" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="F63" s="1" t="s">
+      <c r="F63" s="6" t="s">
         <v>294</v>
       </c>
-      <c r="G63" s="1" t="s">
+      <c r="G63" s="6" t="s">
         <v>295</v>
       </c>
-      <c r="H63" s="1" t="s">
+      <c r="H63" s="6" t="s">
         <v>296</v>
       </c>
-      <c r="I63" s="2" t="s">
+      <c r="I63" s="7" t="s">
         <v>297</v>
       </c>
-      <c r="J63" s="3">
+      <c r="J63" s="20">
         <v>1782</v>
       </c>
-      <c r="K63" s="6">
+      <c r="K63" s="28">
         <v>0.0875</v>
       </c>
     </row>
@@ -4411,7 +4552,7 @@
       <c r="J64" s="3">
         <v>1051</v>
       </c>
-      <c r="K64" s="6">
+      <c r="K64" s="24">
         <v>0.0611111111111111</v>
       </c>
     </row>
@@ -4446,7 +4587,7 @@
       <c r="J65" s="3">
         <v>579</v>
       </c>
-      <c r="K65" s="6">
+      <c r="K65" s="24">
         <v>0.0430555555555556</v>
       </c>
     </row>
@@ -4481,7 +4622,7 @@
       <c r="J66" s="3">
         <v>579</v>
       </c>
-      <c r="K66" s="6">
+      <c r="K66" s="24">
         <v>0.0333333333333333</v>
       </c>
     </row>
@@ -4516,77 +4657,77 @@
       <c r="J67" s="3">
         <v>2285</v>
       </c>
-      <c r="K67" s="6">
+      <c r="K67" s="24">
         <v>0.149305555555556</v>
       </c>
     </row>
     <row r="68" spans="1:11">
-      <c r="A68" s="4">
+      <c r="A68" s="11">
         <v>46086</v>
       </c>
-      <c r="B68" s="1" t="s">
+      <c r="B68" s="12" t="s">
         <v>312</v>
       </c>
-      <c r="C68" s="1" t="s">
+      <c r="C68" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="D68" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E68" s="1" t="s">
+      <c r="D68" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="E68" s="12" t="s">
         <v>313</v>
       </c>
-      <c r="F68" s="1" t="s">
+      <c r="F68" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="G68" s="1" t="s">
+      <c r="G68" s="12" t="s">
         <v>314</v>
       </c>
-      <c r="H68" s="1" t="s">
+      <c r="H68" s="12" t="s">
         <v>315</v>
       </c>
-      <c r="I68" s="2" t="s">
+      <c r="I68" s="13" t="s">
         <v>311</v>
       </c>
-      <c r="J68" s="3">
+      <c r="J68" s="22">
         <v>2576</v>
       </c>
-      <c r="K68" s="6">
+      <c r="K68" s="23">
         <v>0.154861111111111</v>
       </c>
     </row>
     <row r="69" spans="1:11">
-      <c r="A69" s="4">
+      <c r="A69" s="11">
         <v>46089</v>
       </c>
-      <c r="B69" s="1" t="s">
+      <c r="B69" s="12" t="s">
         <v>316</v>
       </c>
-      <c r="C69" s="1" t="s">
+      <c r="C69" s="12" t="s">
         <v>313</v>
       </c>
-      <c r="D69" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E69" s="1" t="s">
+      <c r="D69" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="E69" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="F69" s="1" t="s">
+      <c r="F69" s="12" t="s">
         <v>317</v>
       </c>
-      <c r="G69" s="1" t="s">
+      <c r="G69" s="12" t="s">
         <v>318</v>
       </c>
-      <c r="H69" s="1" t="s">
+      <c r="H69" s="12" t="s">
         <v>319</v>
       </c>
-      <c r="I69" s="2" t="s">
+      <c r="I69" s="13" t="s">
         <v>311</v>
       </c>
-      <c r="J69" s="3">
+      <c r="J69" s="22">
         <v>2576</v>
       </c>
-      <c r="K69" s="6">
+      <c r="K69" s="23">
         <v>0.145138888888889</v>
       </c>
     </row>
@@ -4621,8 +4762,148 @@
       <c r="J70" s="3">
         <v>2285</v>
       </c>
-      <c r="K70" s="6">
+      <c r="K70" s="24">
         <v>0.120138888888889</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11">
+      <c r="A71" s="4">
+        <v>46119</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E71" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="G71" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="H71" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="I71" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="J71" s="3">
+        <v>1051</v>
+      </c>
+      <c r="K71" s="24">
+        <v>0.0659722222222222</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11">
+      <c r="A72" s="4">
+        <v>46120</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E72" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="F72" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="G72" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="H72" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="I72" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="J72" s="3">
+        <v>4960</v>
+      </c>
+      <c r="K72" s="24">
+        <v>0.260416666666667</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11">
+      <c r="A73" s="4">
+        <v>46128</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="C73" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="D73" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E73" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="F73" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G73" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="H73" s="1" t="s">
+        <v>333</v>
+      </c>
+      <c r="I73" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="J73" s="3">
+        <v>3752</v>
+      </c>
+      <c r="K73" s="24">
+        <v>0.1875</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11">
+      <c r="A74" s="4">
+        <v>46128</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="C74" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="D74" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E74" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F74" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="G74" s="1" t="s">
+        <v>336</v>
+      </c>
+      <c r="H74" s="1" t="s">
+        <v>337</v>
+      </c>
+      <c r="I74" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="J74" s="3">
+        <v>579</v>
+      </c>
+      <c r="K74" s="24">
+        <v>0.0402777777777778</v>
       </c>
     </row>
   </sheetData>

</xml_diff>